<commit_message>
Fixing the test name
</commit_message>
<xml_diff>
--- a/src/test/resources/excel/Book2.xlsx
+++ b/src/test/resources/excel/Book2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\F5688728\BongzSeleniumFrameworks\src\test\resources\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9864ECD5-6AAC-4905-B5E6-44A7B21E0670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4467B69-696A-4AA8-AB64-C7802D08556C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{290FA3F8-6C32-43F1-8ED4-F2A44DB688D9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{290FA3F8-6C32-43F1-8ED4-F2A44DB688D9}"/>
   </bookViews>
   <sheets>
     <sheet name="RUNMANAGER" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="48">
   <si>
     <t>testname</t>
   </si>
@@ -161,9 +161,6 @@
   </si>
   <si>
     <t>Miquel507409</t>
-  </si>
-  <si>
-    <t>To check if the advisor can login to platform chat</t>
   </si>
   <si>
     <t>unifiedAgentTest</t>
@@ -606,10 +603,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
@@ -643,7 +640,7 @@
         <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="C6" t="s">
         <v>4</v>
@@ -828,7 +825,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B7" t="s">
         <v>7</v>
@@ -840,10 +837,10 @@
         <v>39</v>
       </c>
       <c r="E7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>45</v>
       </c>
       <c r="G7" t="s">
         <v>25</v>
@@ -860,10 +857,10 @@
         <v>20</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F8" t="s">
         <v>38</v>

</xml_diff>

<commit_message>
Upgrade to Selenium 4 + fix HA shadow DOM login + add Energy navigation
- Upgrade Selenium 3.141.59 to 4.27.0, Java 8 to 11
- Fix HA login: shadow DOM selectors for username/password/submit
- Add HomeAssistantLoginPage with shadow DOM traversal
- Add HomeAssistantDashboardPage with sidebar navigation
- Fix DriverFactory: migrate DesiredCapabilities to browser Options
- Fix ExplicitWaitFactory: Duration-based WebDriverWait, enum comparisons
- Fix MultiplyLoginPage: WaitStrategy.NONE to CLICKABLE/VISIBLE
- Fix BrowserInfoUtils: getVersion() to getBrowserVersion()
- Enable passed step screenshots in config
- Add ExtentReport logging with screenshots to all HA page actions
- Update .gitignore, add README.md
</commit_message>
<xml_diff>
--- a/src/test/resources/excel/Book2.xlsx
+++ b/src/test/resources/excel/Book2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\F5688728\BongzSeleniumFrameworks\src\test\resources\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4467B69-696A-4AA8-AB64-C7802D08556C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84748409-01A9-48BA-BE4D-4135992F1D92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{290FA3F8-6C32-43F1-8ED4-F2A44DB688D9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{290FA3F8-6C32-43F1-8ED4-F2A44DB688D9}"/>
   </bookViews>
   <sheets>
     <sheet name="RUNMANAGER" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="50">
   <si>
     <t>testname</t>
   </si>
@@ -157,9 +157,6 @@
     <t>131.0</t>
   </si>
   <si>
-    <t>advisorLoginToPlatformChatTest</t>
-  </si>
-  <si>
     <t>Miquel507409</t>
   </si>
   <si>
@@ -175,10 +172,19 @@
     <t>To Unified admin</t>
   </si>
   <si>
-    <t>MREOCEP3234617501</t>
-  </si>
-  <si>
     <t>145.0</t>
+  </si>
+  <si>
+    <t>homeAssistantLoginTest</t>
+  </si>
+  <si>
+    <t>To check if the user can successfully login and logout on Home Assistant</t>
+  </si>
+  <si>
+    <t>kbtokzan</t>
+  </si>
+  <si>
+    <t>@KBTokzan2016</t>
   </si>
 </sst>
 </file>
@@ -603,10 +609,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
@@ -637,10 +643,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B6" t="s">
-        <v>3</v>
+        <v>47</v>
       </c>
       <c r="C6" t="s">
         <v>4</v>
@@ -768,7 +774,7 @@
         <v>39</v>
       </c>
       <c r="E4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F4" t="s">
         <v>38</v>
@@ -825,7 +831,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B7" t="s">
         <v>7</v>
@@ -837,10 +843,10 @@
         <v>39</v>
       </c>
       <c r="E7" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>44</v>
       </c>
       <c r="G7" t="s">
         <v>25</v>
@@ -848,7 +854,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
         <v>4</v>
@@ -857,13 +863,13 @@
         <v>20</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E8" t="s">
-        <v>46</v>
-      </c>
-      <c r="F8" t="s">
-        <v>38</v>
+        <v>48</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>29</v>

</xml_diff>